<commit_message>
Normalize result filenames to <input>_<mandate>_<target>[_oil<v>] (no '*', no model name); update in-file references
</commit_message>
<xml_diff>
--- a/results_task_1/claude/1_Y_N_TI_4.xlsx
+++ b/results_task_1/claude/1_Y_N_TI_4.xlsx
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1_Y_N*claude-fable-5.1*TI_4.xlsx</t>
+          <t>1_Y_N_TI_4.xlsx</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1_Y_N*claude-fable-5.1*TI_4.xlsx</t>
+          <t>1_Y_N_TI_4.xlsx</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -635,7 +635,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1_Y_N*claude-fable-5.1*TI_4.xlsx</t>
+          <t>1_Y_N_TI_4.xlsx</t>
         </is>
       </c>
       <c r="B4" t="n">

</xml_diff>